<commit_message>
changes in manage data
</commit_message>
<xml_diff>
--- a/timetable_template.xlsx
+++ b/timetable_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kinda\OneDrive\Desktop\Vorniity\Project MSMe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C486177-9DCD-4956-B258-C413DE7EF43A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F11F6BE-BF92-4F8E-A095-E798D6DBA9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Faculties" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,55 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="236">
+  <si>
+    <t>rule_type</t>
+  </si>
+  <si>
+    <t>subject_codes</t>
+  </si>
+  <si>
+    <t>subject_types</t>
+  </si>
+  <si>
+    <t>period</t>
+  </si>
+  <si>
+    <t>max_period</t>
+  </si>
+  <si>
+    <t>days</t>
+  </si>
+  <si>
+    <t>BEFORE_TIME</t>
+  </si>
+  <si>
+    <t>SOFTSKILL</t>
+  </si>
+  <si>
+    <t>Period 5</t>
+  </si>
+  <si>
+    <t>FIXED_PERIOD</t>
+  </si>
+  <si>
+    <t>OE (Sem 7)</t>
+  </si>
+  <si>
+    <t>Period 3</t>
+  </si>
+  <si>
+    <t>FIXED_DAYS</t>
+  </si>
+  <si>
+    <t>MON, TUE, WED</t>
+  </si>
+  <si>
+    <t>Forum</t>
+  </si>
+  <si>
+    <t>MON</t>
+  </si>
   <si>
     <t>id</t>
   </si>
@@ -204,6 +252,12 @@
     <t>OE Teacher 3 (Sem 7)</t>
   </si>
   <si>
+    <t>MBA</t>
+  </si>
+  <si>
+    <t>MBA Faculty</t>
+  </si>
+  <si>
     <t>code</t>
   </si>
   <si>
@@ -264,9 +318,6 @@
     <t>Big Data Analytics</t>
   </si>
   <si>
-    <t>OE (Sem 7)</t>
-  </si>
-  <si>
     <t>Open Elective (Sem 7)</t>
   </si>
   <si>
@@ -453,18 +504,6 @@
     <t>Mathematics for Lateral Entry Students</t>
   </si>
   <si>
-    <t>NCMC 3</t>
-  </si>
-  <si>
-    <t>NCMC (Sem 3)</t>
-  </si>
-  <si>
-    <t>NCMC 5</t>
-  </si>
-  <si>
-    <t>NCMC (Sem 5)</t>
-  </si>
-  <si>
     <t>LIB_HR</t>
   </si>
   <si>
@@ -492,12 +531,6 @@
     <t>Soft Skills</t>
   </si>
   <si>
-    <t>SOFTSKILL</t>
-  </si>
-  <si>
-    <t>Forum</t>
-  </si>
-  <si>
     <t>semester</t>
   </si>
   <si>
@@ -700,49 +733,13 @@
   </si>
   <si>
     <t>ELEC_3_LAB</t>
-  </si>
-  <si>
-    <t>rule_type</t>
-  </si>
-  <si>
-    <t>subject_codes</t>
-  </si>
-  <si>
-    <t>subject_types</t>
-  </si>
-  <si>
-    <t>period</t>
-  </si>
-  <si>
-    <t>max_period</t>
-  </si>
-  <si>
-    <t>days</t>
-  </si>
-  <si>
-    <t>BEFORE_TIME</t>
-  </si>
-  <si>
-    <t>Period 5</t>
-  </si>
-  <si>
-    <t>FIXED_PERIOD</t>
-  </si>
-  <si>
-    <t>Period 3</t>
-  </si>
-  <si>
-    <t>FIXED_DAYS</t>
-  </si>
-  <si>
-    <t>MON, TUE, WED</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -750,28 +747,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor rgb="FF4472C4"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -779,30 +764,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1105,38 +1072,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="D2">
         <v>6</v>
@@ -1144,13 +1105,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="D3">
         <v>24</v>
@@ -1158,13 +1119,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="D4">
         <v>22</v>
@@ -1172,13 +1133,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D5">
         <v>24</v>
@@ -1186,13 +1147,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D6">
         <v>18</v>
@@ -1200,13 +1161,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D7">
         <v>18</v>
@@ -1214,13 +1175,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D8">
         <v>22</v>
@@ -1228,13 +1189,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D9">
         <v>24</v>
@@ -1242,13 +1203,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D10">
         <v>20</v>
@@ -1256,13 +1217,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D11">
         <v>18</v>
@@ -1270,13 +1231,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D12">
         <v>17</v>
@@ -1284,13 +1245,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
         <v>30</v>
-      </c>
-      <c r="C13" t="s">
-        <v>14</v>
       </c>
       <c r="D13">
         <v>18</v>
@@ -1298,13 +1259,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="D14">
         <v>50</v>
@@ -1312,13 +1273,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D15">
         <v>18</v>
@@ -1326,13 +1287,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D16">
         <v>18</v>
@@ -1340,13 +1301,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D17">
         <v>18</v>
@@ -1354,13 +1315,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D18">
         <v>50</v>
@@ -1368,13 +1329,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D19">
         <v>50</v>
@@ -1382,13 +1343,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="C20" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D20">
         <v>18</v>
@@ -1396,13 +1357,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="C21" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D21">
         <v>18</v>
@@ -1410,13 +1371,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D22">
         <v>50</v>
@@ -1424,13 +1385,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D23">
         <v>18</v>
@@ -1438,13 +1399,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="C24" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D24">
         <v>18</v>
@@ -1452,15 +1413,29 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="C25" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" t="s">
+        <v>30</v>
+      </c>
+      <c r="D26">
         <v>18</v>
       </c>
     </row>
@@ -1473,991 +1448,944 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>63</v>
+      <c r="A1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D2">
         <v>3</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="b">
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" t="b">
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" t="b">
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" t="b">
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D6">
         <v>4</v>
       </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" t="b">
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D7">
         <v>3</v>
       </c>
-      <c r="E7" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" t="b">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
-      <c r="E8" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" t="b">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D9">
         <v>3</v>
       </c>
-      <c r="E9" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" t="b">
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>81</v>
+        <v>98</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D10">
         <v>6</v>
       </c>
-      <c r="E10" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" t="b">
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" t="s">
         <v>84</v>
-      </c>
-      <c r="B11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C11" t="s">
-        <v>66</v>
       </c>
       <c r="D11">
         <v>3</v>
       </c>
-      <c r="E11" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" t="b">
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D12">
         <v>3</v>
       </c>
-      <c r="E12" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" t="b">
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" t="b">
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
-      <c r="E14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" t="b">
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="B15" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" t="b">
-        <v>0</v>
-      </c>
-      <c r="F15" t="b">
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D16">
         <v>4</v>
       </c>
-      <c r="E16" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" t="b">
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="C17" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D17">
         <v>3</v>
       </c>
-      <c r="E17" t="b">
-        <v>0</v>
-      </c>
-      <c r="F17" t="b">
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="B18" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D18">
         <v>6</v>
       </c>
-      <c r="E18" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" t="b">
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="B19" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D19">
         <v>4</v>
       </c>
-      <c r="E19" t="b">
-        <v>1</v>
-      </c>
-      <c r="F19" t="b">
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B20" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D20">
         <v>3</v>
       </c>
-      <c r="E20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F20" t="b">
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="B21" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="E21" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" t="b">
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="B22" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D22">
         <v>5</v>
       </c>
-      <c r="E22" t="b">
-        <v>1</v>
-      </c>
-      <c r="F22" t="b">
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="C23" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D23">
         <v>1</v>
       </c>
-      <c r="E23" t="b">
-        <v>1</v>
-      </c>
-      <c r="F23" t="b">
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="B24" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="C24" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D24">
         <v>1</v>
       </c>
-      <c r="E24" t="b">
-        <v>1</v>
-      </c>
-      <c r="F24" t="b">
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="B25" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="C25" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D25">
         <v>1</v>
       </c>
-      <c r="E25" t="b">
-        <v>1</v>
-      </c>
-      <c r="F25" t="b">
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B26" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D26">
         <v>1</v>
       </c>
-      <c r="E26" t="b">
-        <v>0</v>
-      </c>
-      <c r="F26" t="b">
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="B27" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="C27" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D27">
         <v>1</v>
       </c>
-      <c r="E27" t="b">
-        <v>0</v>
-      </c>
-      <c r="F27" t="b">
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="B28" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="C28" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D28">
         <v>3</v>
       </c>
-      <c r="E28" t="b">
-        <v>0</v>
-      </c>
-      <c r="F28" t="b">
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="B29" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D29">
         <v>3</v>
       </c>
-      <c r="E29" t="b">
-        <v>0</v>
-      </c>
-      <c r="F29" t="b">
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="B30" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D30">
         <v>3</v>
       </c>
-      <c r="E30" t="b">
-        <v>1</v>
-      </c>
-      <c r="F30" t="b">
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="B31" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="C31" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D31">
         <v>3</v>
       </c>
-      <c r="E31" t="b">
-        <v>1</v>
-      </c>
-      <c r="F31" t="b">
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="B32" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D32">
         <v>4</v>
       </c>
-      <c r="E32" t="b">
-        <v>1</v>
-      </c>
-      <c r="F32" t="b">
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="C33" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D33">
         <v>5</v>
       </c>
-      <c r="E33" t="b">
-        <v>1</v>
-      </c>
-      <c r="F33" t="b">
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="C34" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D34">
         <v>3</v>
       </c>
-      <c r="E34" t="b">
-        <v>1</v>
-      </c>
-      <c r="F34" t="b">
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="B35" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="C35" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D35">
         <v>3</v>
       </c>
-      <c r="E35" t="b">
-        <v>1</v>
-      </c>
-      <c r="F35" t="b">
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="B36" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D36">
         <v>1</v>
       </c>
-      <c r="E36" t="b">
-        <v>1</v>
-      </c>
-      <c r="F36" t="b">
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="C37" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D37">
         <v>1</v>
       </c>
-      <c r="E37" t="b">
-        <v>0</v>
-      </c>
-      <c r="F37" t="b">
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="C38" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D38">
         <v>1</v>
       </c>
-      <c r="E38" t="b">
-        <v>0</v>
-      </c>
-      <c r="F38" t="b">
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="B39" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="C39" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D39">
         <v>1</v>
       </c>
-      <c r="E39" t="b">
-        <v>0</v>
-      </c>
-      <c r="F39" t="b">
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39">
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="B40" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="C40" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D40">
         <v>1</v>
       </c>
-      <c r="E40" t="b">
-        <v>1</v>
-      </c>
-      <c r="F40" t="b">
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="B41" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="C41" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D41">
         <v>1</v>
       </c>
-      <c r="E41" t="b">
-        <v>0</v>
-      </c>
-      <c r="F41" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>142</v>
-      </c>
-      <c r="B42" t="s">
-        <v>143</v>
-      </c>
-      <c r="C42" t="s">
-        <v>66</v>
-      </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="E42" t="b">
-        <v>0</v>
-      </c>
-      <c r="F42" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>144</v>
-      </c>
-      <c r="B43" t="s">
-        <v>145</v>
-      </c>
-      <c r="C43" t="s">
-        <v>66</v>
-      </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
-      <c r="E43" t="b">
-        <v>0</v>
-      </c>
-      <c r="F43" t="b">
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
         <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="B44" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C44" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D44">
         <v>1</v>
       </c>
-      <c r="E44" t="b">
-        <v>0</v>
-      </c>
-      <c r="F44" t="b">
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
         <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="B45" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="C45" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D45">
         <v>1</v>
       </c>
-      <c r="E45" t="b">
-        <v>0</v>
-      </c>
-      <c r="F45" t="b">
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="B46" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="C46" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D46">
         <v>1</v>
       </c>
-      <c r="E46" t="b">
-        <v>0</v>
-      </c>
-      <c r="F46" t="b">
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B47" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="C47" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D47">
         <v>1</v>
       </c>
-      <c r="E47" t="b">
-        <v>0</v>
-      </c>
-      <c r="F47" t="b">
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
         <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="B48" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="C48" t="s">
-        <v>155</v>
+        <v>7</v>
       </c>
       <c r="D48">
         <v>1</v>
       </c>
-      <c r="E48" t="b">
-        <v>1</v>
-      </c>
-      <c r="F48" t="b">
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>156</v>
+        <v>14</v>
       </c>
       <c r="B49" t="s">
-        <v>156</v>
+        <v>14</v>
       </c>
       <c r="C49" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="D49">
         <v>1</v>
       </c>
-      <c r="E49" t="b">
-        <v>1</v>
-      </c>
-      <c r="F49" t="b">
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49">
         <v>0</v>
       </c>
     </row>
@@ -2470,28 +2398,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="3" width="12" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>158</v>
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="B2" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C2">
         <v>70</v>
@@ -2499,10 +2423,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="B3" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="C3">
         <v>70</v>
@@ -2510,10 +2434,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="B4" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="C4">
         <v>70</v>
@@ -2521,10 +2445,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="B5" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C5">
         <v>70</v>
@@ -2532,10 +2456,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="C6">
         <v>70</v>
@@ -2543,10 +2467,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="B7" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="C7">
         <v>70</v>
@@ -2554,10 +2478,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="B8" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="C8">
         <v>70</v>
@@ -2565,10 +2489,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="C9">
         <v>70</v>
@@ -2576,10 +2500,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="B10" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="C10">
         <v>70</v>
@@ -2587,10 +2511,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="B11" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="C11">
         <v>70</v>
@@ -2598,10 +2522,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="B12" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C12">
         <v>35</v>
@@ -2609,10 +2533,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="B13" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="C13">
         <v>35</v>
@@ -2620,10 +2544,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="B14" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="C14">
         <v>35</v>
@@ -2631,10 +2555,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="B15" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="C15">
         <v>35</v>
@@ -2642,10 +2566,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>194</v>
+      </c>
+      <c r="B16" t="s">
         <v>183</v>
-      </c>
-      <c r="B16" t="s">
-        <v>172</v>
       </c>
       <c r="C16">
         <v>35</v>
@@ -2653,10 +2577,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="B17" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="C17">
         <v>35</v>
@@ -2664,10 +2588,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="B18" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="C18">
         <v>35</v>
@@ -2675,10 +2599,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="B19" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="C19">
         <v>35</v>
@@ -2686,10 +2610,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="B20" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C20">
         <v>35</v>
@@ -2697,10 +2621,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="B21" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C21">
         <v>35</v>
@@ -2708,10 +2632,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="B22" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="C22">
         <v>35</v>
@@ -2719,10 +2643,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="B23" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="C23">
         <v>35</v>
@@ -2730,10 +2654,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="B24" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="C24">
         <v>35</v>
@@ -2741,10 +2665,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="B25" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="C25">
         <v>35</v>
@@ -2752,10 +2676,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="B26" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="C26">
         <v>35</v>
@@ -2763,10 +2687,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="B27" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="C27">
         <v>35</v>
@@ -2774,10 +2698,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="B28" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="C28">
         <v>35</v>
@@ -2785,10 +2709,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="B29" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="C29">
         <v>35</v>
@@ -2803,30 +2727,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>199</v>
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D1" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="B2">
         <v>75</v>
@@ -2835,12 +2753,12 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="B3">
         <v>75</v>
@@ -2849,12 +2767,12 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="B4">
         <v>75</v>
@@ -2863,12 +2781,12 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="B5">
         <v>75</v>
@@ -2877,12 +2795,12 @@
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="B6">
         <v>75</v>
@@ -2891,12 +2809,12 @@
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="B7">
         <v>75</v>
@@ -2905,12 +2823,12 @@
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="B8">
         <v>75</v>
@@ -2919,12 +2837,12 @@
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="B9">
         <v>75</v>
@@ -2933,12 +2851,12 @@
         <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="B10">
         <v>75</v>
@@ -2947,12 +2865,12 @@
         <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="B11">
         <v>40</v>
@@ -2961,12 +2879,12 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="B12">
         <v>40</v>
@@ -2975,7 +2893,7 @@
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -2985,829 +2903,807 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D140"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>216</v>
+      <c r="A1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D1" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="D4" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="D5" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C6" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="D6" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="D7" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="C9" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="D10" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="C11" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="D11" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="C12" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="D12" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="D13" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C16" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="D16" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="D17" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="C18" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="D18" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="D19" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="D20" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B21" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="C21" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="D21" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="C22" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="C23" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25" t="s">
         <v>10</v>
       </c>
-      <c r="B25" t="s">
-        <v>81</v>
-      </c>
       <c r="C25" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B27" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="C27" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="C28" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="B29" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
-        <v>171</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="C31" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C32" t="s">
-        <v>171</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="B33" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="C33" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="C34" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="B35" t="s">
-        <v>93</v>
+        <v>115</v>
       </c>
       <c r="C35" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C36" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="C37" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="B38" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="C38" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B39" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="C39" t="s">
-        <v>163</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B40" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="C40" t="s">
-        <v>165</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B41" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="C41" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="C42" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B43" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="C43" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B44" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="C44" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="C45" t="s">
-        <v>163</v>
+        <v>196</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="B46" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="C46" t="s">
-        <v>165</v>
+        <v>197</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B47" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="C47" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B48" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="C48" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B49" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="C49" t="s">
-        <v>187</v>
+        <v>174</v>
+      </c>
+      <c r="D49" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B50" t="s">
-        <v>105</v>
+        <v>134</v>
       </c>
       <c r="C50" t="s">
-        <v>188</v>
+        <v>174</v>
+      </c>
+      <c r="D50" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="B51" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="C51" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D51" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B52" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="C52" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D52" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B53" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C53" t="s">
-        <v>165</v>
-      </c>
-      <c r="D53" t="s">
-        <v>222</v>
+        <v>174</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B54" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C54" t="s">
-        <v>165</v>
-      </c>
-      <c r="D54" t="s">
-        <v>222</v>
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="B55" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="C55" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="C56" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="B57" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="C57" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="B58" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="C58" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>47</v>
-      </c>
-      <c r="B59" t="s">
-        <v>113</v>
-      </c>
-      <c r="C59" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>47</v>
-      </c>
-      <c r="B60" t="s">
-        <v>113</v>
-      </c>
-      <c r="C60" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="B61" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="C61" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B62" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="C62" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B63" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="C63" t="s">
-        <v>173</v>
+        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B64" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="C64" t="s">
-        <v>173</v>
+        <v>201</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="B65" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="C65" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="B66" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="C66" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="B67" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="C67" t="s">
-        <v>173</v>
+        <v>201</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="B68" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="C68" t="s">
-        <v>189</v>
+        <v>184</v>
+      </c>
+      <c r="D68" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B69" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
       <c r="C69" t="s">
-        <v>190</v>
+        <v>184</v>
+      </c>
+      <c r="D69" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
@@ -3815,804 +3711,633 @@
         <v>23</v>
       </c>
       <c r="B70" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C70" t="s">
-        <v>173</v>
-      </c>
-      <c r="D70" t="s">
-        <v>223</v>
+        <v>184</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="B71" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C71" t="s">
-        <v>173</v>
-      </c>
-      <c r="D71" t="s">
-        <v>223</v>
+        <v>184</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="B72" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="C72" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>39</v>
-      </c>
-      <c r="B73" t="s">
-        <v>111</v>
-      </c>
-      <c r="C73" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="B74" t="s">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="C74" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="B75" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C75" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B76" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="C76" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B77" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="C77" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B78" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="C78" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B79" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="C79" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="B80" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="C80" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B81" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="C81" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B82" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="C82" t="s">
-        <v>167</v>
+        <v>202</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B83" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="C83" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="B84" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="C84" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B85" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="C85" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="B86" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="C86" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B87" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="C87" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B88" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="C88" t="s">
-        <v>167</v>
+        <v>178</v>
+      </c>
+      <c r="D88" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B89" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="C89" t="s">
-        <v>169</v>
+        <v>180</v>
+      </c>
+      <c r="D89" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="B90" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="C90" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="D90" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="B91" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="C91" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="D91" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B92" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C92" t="s">
-        <v>167</v>
-      </c>
-      <c r="D92" t="s">
-        <v>224</v>
+        <v>178</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B93" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C93" t="s">
-        <v>169</v>
-      </c>
-      <c r="D93" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>12</v>
-      </c>
-      <c r="B94" t="s">
-        <v>138</v>
-      </c>
-      <c r="C94" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>12</v>
-      </c>
-      <c r="B95" t="s">
-        <v>138</v>
-      </c>
-      <c r="C95" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="B96" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="C96" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>21</v>
+        <v>65</v>
       </c>
       <c r="B97" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="C97" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B98" t="s">
         <v>140</v>
       </c>
       <c r="C98" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B99" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C99" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B100" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="C100" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B101" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="C101" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B102" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="C102" t="s">
-        <v>175</v>
+        <v>206</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="B103" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="C103" t="s">
-        <v>175</v>
+        <v>207</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B104" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="C104" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B105" t="s">
-        <v>131</v>
+        <v>151</v>
       </c>
       <c r="C105" t="s">
-        <v>196</v>
+        <v>186</v>
+      </c>
+      <c r="D105" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="B106" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="C106" t="s">
-        <v>175</v>
+        <v>186</v>
+      </c>
+      <c r="D106" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="B107" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="C107" t="s">
-        <v>175</v>
-      </c>
-      <c r="D107" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
-        <v>38</v>
-      </c>
-      <c r="B108" t="s">
-        <v>136</v>
-      </c>
-      <c r="C108" t="s">
-        <v>175</v>
-      </c>
-      <c r="D108" t="s">
-        <v>224</v>
+        <v>186</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="B109" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="C109" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B110" t="s">
-        <v>142</v>
+        <v>14</v>
       </c>
       <c r="C110" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B111" t="s">
-        <v>140</v>
+        <v>14</v>
       </c>
       <c r="C111" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B112" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C112" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B113" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C113" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B114" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C114" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B115" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C115" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B116" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C116" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B117" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C117" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="B118" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C118" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B119" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
       <c r="C119" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B120" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C120" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B121" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C121" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B122" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C122" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B123" t="s">
-        <v>156</v>
+        <v>124</v>
       </c>
       <c r="C123" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B124" t="s">
-        <v>156</v>
+        <v>124</v>
       </c>
       <c r="C124" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B125" t="s">
-        <v>156</v>
+        <v>98</v>
       </c>
       <c r="C125" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B126" t="s">
-        <v>156</v>
+        <v>98</v>
       </c>
       <c r="C126" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B127" t="s">
-        <v>156</v>
+        <v>114</v>
       </c>
       <c r="C127" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="B128" t="s">
-        <v>156</v>
+        <v>82</v>
       </c>
       <c r="C128" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="B129" t="s">
-        <v>156</v>
+        <v>82</v>
       </c>
       <c r="C129" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
-        <v>23</v>
-      </c>
-      <c r="B130" t="s">
-        <v>109</v>
-      </c>
-      <c r="C130" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A131" t="s">
-        <v>10</v>
-      </c>
-      <c r="B131" t="s">
-        <v>138</v>
-      </c>
-      <c r="C131" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A132" t="s">
-        <v>10</v>
-      </c>
-      <c r="B132" t="s">
-        <v>138</v>
-      </c>
-      <c r="C132" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A133" t="s">
-        <v>7</v>
-      </c>
-      <c r="B133" t="s">
-        <v>138</v>
-      </c>
-      <c r="C133" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A134" t="s">
-        <v>12</v>
-      </c>
-      <c r="B134" t="s">
-        <v>107</v>
-      </c>
-      <c r="C134" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A135" t="s">
-        <v>12</v>
-      </c>
-      <c r="B135" t="s">
-        <v>107</v>
-      </c>
-      <c r="C135" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A136" t="s">
-        <v>10</v>
-      </c>
-      <c r="B136" t="s">
-        <v>81</v>
-      </c>
-      <c r="C136" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A137" t="s">
-        <v>12</v>
-      </c>
-      <c r="B137" t="s">
-        <v>81</v>
-      </c>
-      <c r="C137" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A138" t="s">
-        <v>23</v>
-      </c>
-      <c r="B138" t="s">
-        <v>97</v>
-      </c>
-      <c r="C138" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A139" t="s">
-        <v>31</v>
-      </c>
-      <c r="B139" t="s">
-        <v>64</v>
-      </c>
-      <c r="C139" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A140" t="s">
-        <v>31</v>
-      </c>
-      <c r="B140" t="s">
-        <v>64</v>
-      </c>
-      <c r="C140" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -4622,78 +4347,85 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>230</v>
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>231</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>155</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>232</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>233</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>234</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>235</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>236</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>231</v>
-      </c>
-      <c r="C5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" t="s">
-        <v>232</v>
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>